<commit_message>
Integrate mock test into input test into test/mock test by testType, update old data and stream by testType, and fix the error of deleting data that causes the roadmap editing page to not load.
</commit_message>
<xml_diff>
--- a/fe-admin/public/import-samples/sample-placement-test.xlsx
+++ b/fe-admin/public/import-samples/sample-placement-test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="11460"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="137">
   <si>
     <t>Field</t>
   </si>
@@ -53,6 +53,12 @@
   </si>
   <si>
     <t>Reading</t>
+  </si>
+  <si>
+    <t>testtype</t>
+  </si>
+  <si>
+    <t>checkpoint</t>
   </si>
   <si>
     <t>TimeLimit</t>
@@ -1519,8 +1525,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" outlineLevelRow="5" outlineLevelCol="1"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" outlineLevelRow="6" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="12.25" style="10" customWidth="1"/>
     <col min="2" max="2" width="53.75" style="11" customWidth="1"/>
@@ -1563,23 +1569,31 @@
       <c r="A5" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" ht="33.75" customHeight="1" spans="1:2">
+      <c r="A6" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="9">
         <v>60</v>
       </c>
     </row>
-    <row r="6" ht="57" customHeight="1" spans="1:2">
-      <c r="A6" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>10</v>
+    <row r="7" ht="57" customHeight="1" spans="1:2">
+      <c r="A7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A4 A5:B6 A1:B3" numberStoredAsText="1"/>
+    <ignoredError sqref="B1 A2:B3 A6:B7 A4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1596,13 +1610,13 @@
   <sheetData>
     <row r="1" customHeight="1" spans="1:5">
       <c r="A1" s="7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
@@ -1612,16 +1626,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" ht="182.25" customHeight="1" spans="1:5">
@@ -1629,16 +1643,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" ht="182.25" customHeight="1" spans="1:5">
@@ -1646,23 +1660,23 @@
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 A2:E4" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:E4 A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1688,34 +1702,34 @@
   <sheetData>
     <row r="1" customHeight="1" spans="1:10">
       <c r="A1" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:10">
@@ -1726,28 +1740,28 @@
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E2" s="5">
         <v>1</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" customHeight="1" spans="1:10">
@@ -1758,28 +1772,28 @@
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="5">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="5">
-        <v>1</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>32</v>
-      </c>
       <c r="I3" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" customHeight="1" spans="1:10">
@@ -1790,28 +1804,28 @@
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E4" s="5">
         <v>1</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" customHeight="1" spans="1:10">
@@ -1822,28 +1836,28 @@
         <v>0</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E5" s="5">
         <v>1</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" customHeight="1" spans="1:10">
@@ -1854,28 +1868,28 @@
         <v>0</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E6" s="5">
         <v>1</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7" customHeight="1" spans="1:10">
@@ -1886,28 +1900,28 @@
         <v>0</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E7" s="5">
         <v>1</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="1:10">
@@ -1918,28 +1932,28 @@
         <v>0</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" customHeight="1" spans="1:10">
@@ -1950,28 +1964,28 @@
         <v>0</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E9" s="5">
         <v>1</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="1:10">
@@ -1982,28 +1996,28 @@
         <v>0</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="1:10">
@@ -2014,28 +2028,28 @@
         <v>0</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E11" s="5">
         <v>1</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="1:10">
@@ -2046,28 +2060,28 @@
         <v>1</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E12" s="5">
         <v>1</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="1:10">
@@ -2078,28 +2092,28 @@
         <v>1</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" customHeight="1" spans="1:10">
@@ -2110,28 +2124,28 @@
         <v>1</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E14" s="5">
         <v>1</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" customHeight="1" spans="1:10">
@@ -2142,28 +2156,28 @@
         <v>1</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E15" s="5">
         <v>1</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="1:10">
@@ -2174,28 +2188,28 @@
         <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E16" s="5">
         <v>1</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="1:10">
@@ -2206,28 +2220,28 @@
         <v>1</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E17" s="5">
         <v>1</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="1:10">
@@ -2238,28 +2252,28 @@
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E18" s="5">
         <v>1</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="19" customHeight="1" spans="1:10">
@@ -2270,28 +2284,28 @@
         <v>1</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E19" s="5">
         <v>1</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" customHeight="1" spans="1:10">
@@ -2302,28 +2316,28 @@
         <v>1</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E20" s="5">
         <v>1</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:10">
@@ -2334,28 +2348,28 @@
         <v>1</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E21" s="5">
         <v>1</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="1:10">
@@ -2366,28 +2380,28 @@
         <v>2</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E22" s="5">
         <v>1</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" customHeight="1" spans="1:10">
@@ -2398,28 +2412,28 @@
         <v>2</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E23" s="5">
         <v>1</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="1:10">
@@ -2430,28 +2444,28 @@
         <v>2</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E24" s="5">
         <v>1</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" customHeight="1" spans="1:10">
@@ -2462,28 +2476,28 @@
         <v>2</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E25" s="5">
         <v>1</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" customHeight="1" spans="1:10">
@@ -2494,28 +2508,28 @@
         <v>2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E26" s="5">
         <v>1</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="1:10">
@@ -2526,28 +2540,28 @@
         <v>2</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E27" s="5">
         <v>1</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="1:10">
@@ -2558,28 +2572,28 @@
         <v>2</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E28" s="5">
         <v>1</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="1:10">
@@ -2590,28 +2604,28 @@
         <v>2</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E29" s="5">
         <v>1</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:10">
@@ -2622,28 +2636,28 @@
         <v>2</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E30" s="5">
         <v>1</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" customHeight="1" spans="1:10">
@@ -2654,28 +2668,28 @@
         <v>2</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E31" s="5">
         <v>1</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J31" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" customHeight="1" spans="1:10">
@@ -2686,28 +2700,28 @@
         <v>2</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E32" s="5">
         <v>1</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" customHeight="1" spans="1:10">
@@ -2718,28 +2732,28 @@
         <v>2</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E33" s="5">
         <v>1</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J33" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" customHeight="1" spans="1:10">
@@ -2750,28 +2764,28 @@
         <v>2</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E34" s="5">
         <v>1</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="35" customHeight="1" spans="1:10">
@@ -2782,28 +2796,28 @@
         <v>2</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E35" s="5">
         <v>1</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix backend delete point
</commit_message>
<xml_diff>
--- a/fe-admin/public/import-samples/sample-placement-test.xlsx
+++ b/fe-admin/public/import-samples/sample-placement-test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9000"/>
+    <workbookView windowWidth="22188" windowHeight="9000" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="136">
   <si>
     <t>Field</t>
   </si>
@@ -113,9 +113,6 @@
   </si>
   <si>
     <t>Content</t>
-  </si>
-  <si>
-    <t>Points</t>
   </si>
   <si>
     <t>AllowMultiple</t>
@@ -1593,7 +1590,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="B1 A2:B3 A6:B7 A4" numberStoredAsText="1"/>
+    <ignoredError sqref="A4 A6:B7 A2:B3 B1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1676,7 +1673,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A2:E4 A1:C1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1 A2:E4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1684,23 +1681,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="25.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.25" style="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
     <col min="4" max="4" width="61" style="2" customWidth="1"/>
-    <col min="5" max="5" width="6.75" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.75" style="1" customWidth="1"/>
-    <col min="7" max="7" width="27.25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="55.875" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="1"/>
+    <col min="5" max="5" width="13.75" style="1" customWidth="1"/>
+    <col min="6" max="6" width="27.25" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="55.875" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:10">
+    <row r="1" customHeight="1" spans="1:9">
       <c r="A1" s="3" t="s">
         <v>22</v>
       </c>
@@ -1725,14 +1721,11 @@
       <c r="H1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:10">
+    </row>
+    <row r="2" customHeight="1" spans="1:9">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1740,31 +1733,28 @@
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>32</v>
-      </c>
-      <c r="E2" s="5">
-        <v>1</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" customHeight="1" spans="1:10">
+    </row>
+    <row r="3" customHeight="1" spans="1:9">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1772,31 +1762,28 @@
         <v>0</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="5">
-        <v>1</v>
+        <v>35</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:9">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1804,31 +1791,28 @@
         <v>0</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E4" s="5">
-        <v>1</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>39</v>
       </c>
       <c r="H4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="5" customHeight="1" spans="1:10">
+    </row>
+    <row r="5" customHeight="1" spans="1:9">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1836,31 +1820,28 @@
         <v>0</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="5">
-        <v>1</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" customHeight="1" spans="1:10">
+    </row>
+    <row r="6" customHeight="1" spans="1:9">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1868,31 +1849,28 @@
         <v>0</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="5">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="7" customHeight="1" spans="1:10">
+    </row>
+    <row r="7" customHeight="1" spans="1:9">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1900,31 +1878,28 @@
         <v>0</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="E7" s="5">
-        <v>1</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>50</v>
       </c>
       <c r="H7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" customHeight="1" spans="1:10">
+    </row>
+    <row r="8" customHeight="1" spans="1:9">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -1932,31 +1907,28 @@
         <v>0</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="E8" s="5">
-        <v>1</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>54</v>
       </c>
       <c r="H8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" customHeight="1" spans="1:10">
+    </row>
+    <row r="9" customHeight="1" spans="1:9">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -1964,31 +1936,28 @@
         <v>0</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="5">
-        <v>1</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" customHeight="1" spans="1:10">
+    </row>
+    <row r="10" customHeight="1" spans="1:9">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -1996,31 +1965,28 @@
         <v>0</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="5">
-        <v>1</v>
+        <v>59</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" customHeight="1" spans="1:9">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -2028,31 +1994,28 @@
         <v>0</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="E11" s="5">
-        <v>1</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>63</v>
       </c>
       <c r="H11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="I11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" customHeight="1" spans="1:10">
+    </row>
+    <row r="12" customHeight="1" spans="1:9">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -2060,31 +2023,28 @@
         <v>1</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="E12" s="5">
-        <v>1</v>
+        <v>65</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I12" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" customHeight="1" spans="1:9">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -2092,31 +2052,28 @@
         <v>1</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="E13" s="5">
-        <v>1</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>69</v>
       </c>
       <c r="H13" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I13" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" customHeight="1" spans="1:10">
+    </row>
+    <row r="14" customHeight="1" spans="1:9">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -2124,31 +2081,28 @@
         <v>1</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E14" s="5">
-        <v>1</v>
+        <v>71</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" customHeight="1" spans="1:9">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -2156,31 +2110,28 @@
         <v>1</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D15" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="5">
-        <v>1</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="I15" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16" customHeight="1" spans="1:10">
+    </row>
+    <row r="16" customHeight="1" spans="1:9">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -2188,31 +2139,28 @@
         <v>1</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D16" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="E16" s="5">
-        <v>1</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>78</v>
       </c>
       <c r="H16" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="I16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="17" customHeight="1" spans="1:10">
+    </row>
+    <row r="17" customHeight="1" spans="1:9">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -2220,31 +2168,28 @@
         <v>1</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="E17" s="5">
-        <v>1</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>82</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="I17" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="18" customHeight="1" spans="1:10">
+    </row>
+    <row r="18" customHeight="1" spans="1:9">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -2252,31 +2197,28 @@
         <v>1</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D18" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E18" s="5">
-        <v>1</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="I18" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="19" customHeight="1" spans="1:10">
+    </row>
+    <row r="19" customHeight="1" spans="1:9">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -2284,31 +2226,28 @@
         <v>1</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E19" s="5">
-        <v>1</v>
+        <v>87</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>78</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" customHeight="1" spans="1:9">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -2316,31 +2255,28 @@
         <v>1</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D20" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="E20" s="5">
-        <v>1</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>91</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="I20" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="21" customHeight="1" spans="1:10">
+    </row>
+    <row r="21" customHeight="1" spans="1:9">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -2348,31 +2284,28 @@
         <v>1</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="E21" s="5">
-        <v>1</v>
+        <v>93</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>39</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" customHeight="1" spans="1:9">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -2380,31 +2313,28 @@
         <v>2</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="E22" s="5">
-        <v>1</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>97</v>
       </c>
       <c r="H22" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="I22" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J22" s="6" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="23" customHeight="1" spans="1:10">
+    </row>
+    <row r="23" customHeight="1" spans="1:9">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -2412,31 +2342,28 @@
         <v>2</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D23" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E23" s="5">
-        <v>1</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I23" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="I23" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J23" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="24" customHeight="1" spans="1:10">
+    </row>
+    <row r="24" customHeight="1" spans="1:9">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -2444,31 +2371,28 @@
         <v>2</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D24" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="E24" s="5">
-        <v>1</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>104</v>
       </c>
       <c r="H24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I24" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="I24" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J24" s="6" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="25" customHeight="1" spans="1:10">
+    </row>
+    <row r="25" customHeight="1" spans="1:9">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -2476,31 +2400,28 @@
         <v>2</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E25" s="5">
-        <v>1</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="I25" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="26" customHeight="1" spans="1:10">
+    </row>
+    <row r="26" customHeight="1" spans="1:9">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -2508,31 +2429,28 @@
         <v>2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E26" s="5">
-        <v>1</v>
+        <v>109</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J26" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="27" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" customHeight="1" spans="1:9">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -2540,31 +2458,28 @@
         <v>2</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D27" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E27" s="5">
-        <v>1</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="I27" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J27" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="28" customHeight="1" spans="1:10">
+    </row>
+    <row r="28" customHeight="1" spans="1:9">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -2572,31 +2487,28 @@
         <v>2</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="E28" s="5">
-        <v>1</v>
+        <v>114</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G28" s="5" t="s">
         <v>33</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J28" s="6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="29" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" customHeight="1" spans="1:9">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -2604,31 +2516,28 @@
         <v>2</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D29" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" s="5" t="s">
         <v>117</v>
-      </c>
-      <c r="E29" s="5">
-        <v>1</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>118</v>
       </c>
       <c r="H29" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="I29" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="30" customHeight="1" spans="1:10">
+    </row>
+    <row r="30" customHeight="1" spans="1:9">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -2636,31 +2545,28 @@
         <v>2</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E30" s="5">
-        <v>1</v>
+        <v>120</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>39</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J30" s="6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="31" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" customHeight="1" spans="1:9">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -2668,31 +2574,28 @@
         <v>2</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D31" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E31" s="5">
-        <v>1</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I31" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="I31" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J31" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="32" customHeight="1" spans="1:10">
+    </row>
+    <row r="32" customHeight="1" spans="1:9">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -2700,31 +2603,28 @@
         <v>2</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="E32" s="5">
-        <v>1</v>
+        <v>125</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>39</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J32" s="6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="33" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" customHeight="1" spans="1:9">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -2732,31 +2632,28 @@
         <v>2</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D33" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="E33" s="5">
-        <v>1</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>129</v>
       </c>
       <c r="H33" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I33" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="I33" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J33" s="6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="34" customHeight="1" spans="1:10">
+    </row>
+    <row r="34" customHeight="1" spans="1:9">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -2764,31 +2661,28 @@
         <v>2</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="E34" s="5">
-        <v>1</v>
+        <v>131</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>39</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="I34" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="35" customHeight="1" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" customHeight="1" spans="1:9">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -2796,35 +2690,32 @@
         <v>2</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D35" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="E35" s="5">
-        <v>1</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="H35" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I35" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="I35" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J35" s="6" t="s">
-        <v>136</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J35" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I35" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>